<commit_message>
Use cost-core 2.7.0, with the CER and phasing examples and an AoA status quo
</commit_message>
<xml_diff>
--- a/examples/aoa.xlsx
+++ b/examples/aoa.xlsx
@@ -427,10 +427,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
   </cols>
@@ -455,11 +455,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Upgrade in place</t>
+          <t>Keep current system</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.62</v>
+        <v>0.4</v>
       </c>
       <c r="C2" t="n">
         <v>0.3</v>
@@ -468,26 +468,39 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>New development</t>
+          <t>Upgrade in place</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9</v>
+        <v>0.62</v>
       </c>
       <c r="C3" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>New development</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>Buy commercial</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B5" t="n">
         <v>0.55</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C5" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -502,11 +515,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -596,33 +609,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Upgrade in place</t>
+          <t>Keep current system</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Development</t>
+          <t>Obsolescence fixes</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>RDT&amp;E</t>
+          <t>Procurement</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="E2" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="F2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>bell</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
@@ -633,39 +642,39 @@
         <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Upgrade in place</t>
+          <t>Keep current system</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Mod kits</t>
+          <t>Operations and support</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Procurement</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2029</v>
-      </c>
-      <c r="F3" t="n">
-        <v>5</v>
-      </c>
+          <t>O&amp;S</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>400</v>
+      </c>
+      <c r="I3" t="n">
+        <v>2027</v>
+      </c>
+      <c r="J3" t="n">
+        <v>2045</v>
+      </c>
       <c r="K3" t="n">
         <v>0.95</v>
       </c>
@@ -673,7 +682,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="N3" t="inlineStr"/>
     </row>
@@ -685,7 +694,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Operations and support</t>
+          <t>Current system until replaced</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -698,29 +707,29 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>260</v>
+        <v>400</v>
       </c>
       <c r="I4" t="n">
-        <v>2030</v>
+        <v>2027</v>
       </c>
       <c r="J4" t="n">
-        <v>2045</v>
+        <v>2029</v>
       </c>
       <c r="K4" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>New development</t>
+          <t>Upgrade in place</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -734,13 +743,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2400</v>
+        <v>600</v>
       </c>
       <c r="E5" t="n">
         <v>2027</v>
       </c>
       <c r="F5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -757,19 +766,19 @@
         <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>New development</t>
+          <t>Upgrade in place</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Mod kits</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -778,13 +787,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4200</v>
+        <v>1500</v>
       </c>
       <c r="E6" t="n">
-        <v>2032</v>
+        <v>2029</v>
       </c>
       <c r="F6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
@@ -797,14 +806,14 @@
         <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>New development</t>
+          <t>Upgrade in place</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -822,22 +831,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>150</v>
+        <v>260</v>
       </c>
       <c r="I7" t="n">
-        <v>2034</v>
+        <v>2030</v>
       </c>
       <c r="J7" t="n">
-        <v>2060</v>
+        <v>2045</v>
       </c>
       <c r="K7" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="N7" t="inlineStr"/>
     </row>
@@ -849,35 +858,47 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Disposal</t>
+          <t>Current system until replaced</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Disposal</t>
+          <t>O&amp;S</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>400</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="J8" t="n">
+        <v>2033</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>1.5</v>
+      </c>
       <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Buy commercial</t>
+          <t>New development</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Development</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -886,15 +907,19 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>300</v>
+        <v>2400</v>
       </c>
       <c r="E9" t="n">
         <v>2027</v>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>bell</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
@@ -905,19 +930,19 @@
         <v>1</v>
       </c>
       <c r="M9" t="n">
-        <v>1.3</v>
+        <v>1.8</v>
       </c>
       <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Buy commercial</t>
+          <t>New development</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Purchase</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -926,13 +951,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2600</v>
+        <v>4200</v>
       </c>
       <c r="E10" t="n">
-        <v>2028</v>
+        <v>2032</v>
       </c>
       <c r="F10" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
@@ -945,14 +970,14 @@
         <v>1</v>
       </c>
       <c r="M10" t="n">
-        <v>1.15</v>
+        <v>1.4</v>
       </c>
       <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Buy commercial</t>
+          <t>New development</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -970,16 +995,16 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>230</v>
+        <v>150</v>
       </c>
       <c r="I11" t="n">
-        <v>2030</v>
+        <v>2034</v>
       </c>
       <c r="J11" t="n">
-        <v>2050</v>
+        <v>2060</v>
       </c>
       <c r="K11" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="L11" t="n">
         <v>1</v>
@@ -988,6 +1013,194 @@
         <v>1.3</v>
       </c>
       <c r="N11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>New development</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Disposal</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Disposal</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Buy commercial</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Current system until replaced</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>O&amp;S</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="n">
+        <v>400</v>
+      </c>
+      <c r="I13" t="n">
+        <v>2027</v>
+      </c>
+      <c r="J13" t="n">
+        <v>2029</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Buy commercial</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>RDT&amp;E</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>300</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2027</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Buy commercial</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Purchase</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>2600</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F15" t="n">
+        <v>5</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="N15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Buy commercial</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Operations and support</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>O&amp;S</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>230</v>
+      </c>
+      <c r="I16" t="n">
+        <v>2030</v>
+      </c>
+      <c r="J16" t="n">
+        <v>2050</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="L16" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1056,7 +1269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1132,32 +1345,44 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Iterations</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>20000</v>
+          <t>Status Quo</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Keep current system</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Iterations</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>7</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Invented numbers, for illustration only: three ways to replace an ageing sensor, in BY2026 $M.</t>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Invented numbers, for illustration only: three ways to replace an ageing sensor, and keeping it, in BY2026 $M.</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1448,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>One cost line per row, naming its Alternative. Give its cost one of three ways: a Total spread over Years from a Start Year (Profile uniform, or bell); an Annual Amount from a First Year to a Last Year; or a row on the Phased sheet with the amount in each year.</t>
+          <t>One cost line per row, naming its Alternative. Give its cost one of three ways: a Total spread over Years from a Start Year (Profile uniform, front, back or bell); an Annual Amount from a First Year to a Last Year; or a row on the Phased sheet with the amount in each year.</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1472,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Base Year is the constant-dollar year. Discount Rate and Inflation Rate are annual (0.02 for 2%). Basis is by, ty or pv: which dollars to compare on.</t>
+          <t>Base Year is the constant-dollar year. Discount Rate and Inflation Rate are annual (0.02 for 2%). Basis is by, ty or pv: which dollars to compare on. Status Quo names the alternative the others are measured against in the economic analysis: what each costs up front, what it saves, whether it pays back and when.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Examples from the styled 2.8.0 templates, and the window in the README
</commit_message>
<xml_diff>
--- a/examples/aoa.xlsx
+++ b/examples/aoa.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,16 +32,52 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F1F1F"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000000"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -49,11 +85,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -62,6 +112,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -136,6 +195,191 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>cost-core</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Required. Each alternative's name, once. The status quo is one of them.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Optional score, on any scale the same for all.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. How much its cost lines overrun together (0.3 if blank).</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>cost-core</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Required. Which alternative the line belongs to.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Required. The cost line, e.g. Development.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Required. RDT&amp;E, Procurement, MILCON, O&amp;S or Disposal.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Way 1: a total spread over Years from Start Year.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Way 1: the first year of the spread.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Way 1: how many years.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Way 1: uniform, front, back or bell.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Way 2: the same amount every year from First Year to Last Year.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Way 2: the first year.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Way 2: the last year.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Uncertainty: e.g. 0.9 means 10% under. Blank for none.</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Uncertainty: usually 1.0.</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Uncertainty: e.g. 1.4 means 40% over.</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. triangular (default), pert or uniform.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>cost-core</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Required. Way 3: the alternative of a line costed year by year.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Required. Way 3: the line, as named on the Lines sheet.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. That fiscal year's cost, in base-year dollars.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. That fiscal year's cost, in base-year dollars.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>cost-core</author>
+  </authors>
+  <commentList>
+    <comment ref="A2" authorId="0" shapeId="0">
+      <text>
+        <t>The dollar year the cost lines are in.</t>
+      </text>
+    </comment>
+    <comment ref="A3" authorId="0" shapeId="0">
+      <text>
+        <t>Real discount rate from OMB A-94: 0.02 for 2%.</t>
+      </text>
+    </comment>
+    <comment ref="A4" authorId="0" shapeId="0">
+      <text>
+        <t>Annual inflation for then-year dollars: 0.02 for 2%.</t>
+      </text>
+    </comment>
+    <comment ref="A5" authorId="0" shapeId="0">
+      <text>
+        <t>What the costs are in, e.g. BY2026 $M.</t>
+      </text>
+    </comment>
+    <comment ref="A6" authorId="0" shapeId="0">
+      <text>
+        <t>pv (present value, the A-94 comparison), by or ty.</t>
+      </text>
+    </comment>
+    <comment ref="A7" authorId="0" shapeId="0">
+      <text>
+        <t>The alternative the others are measured against: investment, savings, payback.</t>
+      </text>
+    </comment>
+    <comment ref="A8" authorId="0" shapeId="0">
+      <text>
+        <t>How many simulations per alternative.</t>
+      </text>
+    </comment>
+    <comment ref="A9" authorId="0" shapeId="0">
+      <text>
+        <t>Any whole number; the same seed gives the same answer.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -424,10 +668,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FFC000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -436,86 +681,213 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Alternative</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Effectiveness</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Correlation</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Keep current system</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="6" t="n">
         <v>0.4</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="6" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Upgrade in place</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="6" t="n">
         <v>0.62</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="6" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>New development</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="6" t="n">
         <v>0.9</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="6" t="n">
         <v>0.4</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Buy commercial</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="6" t="n">
         <v>0.55</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="6" t="n">
         <v>0.2</v>
       </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="6" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="6" t="n"/>
+      <c r="C26" s="6" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="6" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n"/>
+      <c r="B28" s="6" t="n"/>
+      <c r="C28" s="6" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n"/>
+      <c r="B29" s="6" t="n"/>
+      <c r="C29" s="6" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n"/>
+      <c r="B30" s="6" t="n"/>
+      <c r="C30" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FFC000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -535,685 +907,1101 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Alternative</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Line</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Start Year</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Years</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Profile</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Annual Amount</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>First Year</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>Last Year</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>Low Factor</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>Most Likely Factor</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="5" t="inlineStr">
         <is>
           <t>High Factor</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="5" t="inlineStr">
         <is>
           <t>Distribution</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Keep current system</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Obsolescence fixes</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Procurement</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="6" t="n">
         <v>900</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="6" t="n">
         <v>2028</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="n">
+      <c r="G2" s="6" t="inlineStr"/>
+      <c r="H2" s="6" t="inlineStr"/>
+      <c r="I2" s="6" t="inlineStr"/>
+      <c r="J2" s="6" t="inlineStr"/>
+      <c r="K2" s="6" t="n">
         <v>0.9</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M2" s="6" t="n">
         <v>1.6</v>
       </c>
-      <c r="N2" t="inlineStr"/>
+      <c r="N2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Keep current system</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Operations and support</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>O&amp;S</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="n">
+      <c r="D3" s="6" t="inlineStr"/>
+      <c r="E3" s="6" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr"/>
+      <c r="G3" s="6" t="inlineStr"/>
+      <c r="H3" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="6" t="n">
         <v>2027</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="6" t="n">
         <v>2045</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" s="6" t="n">
         <v>0.95</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L3" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M3" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="N3" t="inlineStr"/>
+      <c r="N3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Upgrade in place</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Current system until replaced</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>O&amp;S</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="n">
+      <c r="D4" s="6" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+      <c r="H4" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="6" t="n">
         <v>2027</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J4" s="6" t="n">
         <v>2029</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" s="6" t="n">
         <v>0.95</v>
       </c>
-      <c r="L4" t="n">
+      <c r="L4" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M4" t="n">
+      <c r="M4" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="N4" t="inlineStr"/>
+      <c r="N4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Upgrade in place</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Development</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>RDT&amp;E</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="6" t="n">
         <v>600</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="6" t="n">
         <v>2027</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>bell</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="n">
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="inlineStr"/>
+      <c r="K5" s="6" t="n">
         <v>0.9</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M5" t="n">
+      <c r="M5" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="N5" t="inlineStr"/>
+      <c r="N5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Upgrade in place</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Mod kits</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Procurement</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="6" t="n">
         <v>1500</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="6" t="n">
         <v>2029</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="n">
+      <c r="G6" s="6" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="inlineStr"/>
+      <c r="K6" s="6" t="n">
         <v>0.95</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M6" t="n">
+      <c r="M6" s="6" t="n">
         <v>1.3</v>
       </c>
-      <c r="N6" t="inlineStr"/>
+      <c r="N6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Upgrade in place</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Operations and support</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>O&amp;S</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="n">
+      <c r="D7" s="6" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr"/>
+      <c r="H7" s="6" t="n">
         <v>260</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7" s="6" t="n">
         <v>2030</v>
       </c>
-      <c r="J7" t="n">
+      <c r="J7" s="6" t="n">
         <v>2045</v>
       </c>
-      <c r="K7" t="n">
+      <c r="K7" s="6" t="n">
         <v>0.9</v>
       </c>
-      <c r="L7" t="n">
+      <c r="L7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M7" t="n">
+      <c r="M7" s="6" t="n">
         <v>1.4</v>
       </c>
-      <c r="N7" t="inlineStr"/>
+      <c r="N7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>New development</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Current system until replaced</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>O&amp;S</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="n">
+      <c r="D8" s="6" t="inlineStr"/>
+      <c r="E8" s="6" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr"/>
+      <c r="G8" s="6" t="inlineStr"/>
+      <c r="H8" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I8" s="6" t="n">
         <v>2027</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J8" s="6" t="n">
         <v>2033</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K8" s="6" t="n">
         <v>0.95</v>
       </c>
-      <c r="L8" t="n">
+      <c r="L8" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M8" t="n">
+      <c r="M8" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="N8" t="inlineStr"/>
+      <c r="N8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>New development</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Development</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>RDT&amp;E</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="6" t="n">
         <v>2400</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="6" t="n">
         <v>2027</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>bell</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="n">
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="n">
         <v>0.9</v>
       </c>
-      <c r="L9" t="n">
+      <c r="L9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M9" t="n">
+      <c r="M9" s="6" t="n">
         <v>1.8</v>
       </c>
-      <c r="N9" t="inlineStr"/>
+      <c r="N9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>New development</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Procurement</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="6" t="n">
         <v>4200</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="6" t="n">
         <v>2032</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="n">
+      <c r="G10" s="6" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr"/>
+      <c r="K10" s="6" t="n">
         <v>0.95</v>
       </c>
-      <c r="L10" t="n">
+      <c r="L10" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M10" t="n">
+      <c r="M10" s="6" t="n">
         <v>1.4</v>
       </c>
-      <c r="N10" t="inlineStr"/>
+      <c r="N10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>New development</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Operations and support</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>O&amp;S</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="n">
+      <c r="D11" s="6" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr"/>
+      <c r="G11" s="6" t="inlineStr"/>
+      <c r="H11" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="I11" t="n">
+      <c r="I11" s="6" t="n">
         <v>2034</v>
       </c>
-      <c r="J11" t="n">
+      <c r="J11" s="6" t="n">
         <v>2060</v>
       </c>
-      <c r="K11" t="n">
+      <c r="K11" s="6" t="n">
         <v>0.85</v>
       </c>
-      <c r="L11" t="n">
+      <c r="L11" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M11" t="n">
+      <c r="M11" s="6" t="n">
         <v>1.3</v>
       </c>
-      <c r="N11" t="inlineStr"/>
+      <c r="N11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>New development</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Disposal</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Disposal</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
+      <c r="D12" s="6" t="inlineStr"/>
+      <c r="E12" s="6" t="inlineStr"/>
+      <c r="F12" s="6" t="inlineStr"/>
+      <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr"/>
+      <c r="J12" s="6" t="inlineStr"/>
+      <c r="K12" s="6" t="inlineStr"/>
+      <c r="L12" s="6" t="inlineStr"/>
+      <c r="M12" s="6" t="inlineStr"/>
+      <c r="N12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Buy commercial</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Current system until replaced</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>O&amp;S</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="n">
+      <c r="D13" s="6" t="inlineStr"/>
+      <c r="E13" s="6" t="inlineStr"/>
+      <c r="F13" s="6" t="inlineStr"/>
+      <c r="G13" s="6" t="inlineStr"/>
+      <c r="H13" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="I13" t="n">
+      <c r="I13" s="6" t="n">
         <v>2027</v>
       </c>
-      <c r="J13" t="n">
+      <c r="J13" s="6" t="n">
         <v>2029</v>
       </c>
-      <c r="K13" t="n">
+      <c r="K13" s="6" t="n">
         <v>0.95</v>
       </c>
-      <c r="L13" t="n">
+      <c r="L13" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M13" t="n">
+      <c r="M13" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="N13" t="inlineStr"/>
+      <c r="N13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Buy commercial</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Integration</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>RDT&amp;E</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="6" t="n">
         <v>300</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14" s="6" t="n">
         <v>2027</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="n">
+      <c r="G14" s="6" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr"/>
+      <c r="J14" s="6" t="inlineStr"/>
+      <c r="K14" s="6" t="n">
         <v>0.9</v>
       </c>
-      <c r="L14" t="n">
+      <c r="L14" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M14" t="n">
+      <c r="M14" s="6" t="n">
         <v>1.3</v>
       </c>
-      <c r="N14" t="inlineStr"/>
+      <c r="N14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Buy commercial</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Purchase</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Procurement</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" s="6" t="n">
         <v>2600</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="6" t="n">
         <v>2028</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="n">
+      <c r="G15" s="6" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr"/>
+      <c r="K15" s="6" t="n">
         <v>0.95</v>
       </c>
-      <c r="L15" t="n">
+      <c r="L15" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M15" t="n">
+      <c r="M15" s="6" t="n">
         <v>1.15</v>
       </c>
-      <c r="N15" t="inlineStr"/>
+      <c r="N15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Buy commercial</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Operations and support</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>O&amp;S</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="n">
+      <c r="D16" s="6" t="inlineStr"/>
+      <c r="E16" s="6" t="inlineStr"/>
+      <c r="F16" s="6" t="inlineStr"/>
+      <c r="G16" s="6" t="inlineStr"/>
+      <c r="H16" s="6" t="n">
         <v>230</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I16" s="6" t="n">
         <v>2030</v>
       </c>
-      <c r="J16" t="n">
+      <c r="J16" s="6" t="n">
         <v>2050</v>
       </c>
-      <c r="K16" t="n">
+      <c r="K16" s="6" t="n">
         <v>0.9</v>
       </c>
-      <c r="L16" t="n">
+      <c r="L16" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M16" t="n">
+      <c r="M16" s="6" t="n">
         <v>1.3</v>
       </c>
-      <c r="N16" t="inlineStr"/>
+      <c r="N16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="6" t="n"/>
+      <c r="L17" s="6" t="n"/>
+      <c r="M17" s="6" t="n"/>
+      <c r="N17" s="6" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+      <c r="I18" s="6" t="n"/>
+      <c r="J18" s="6" t="n"/>
+      <c r="K18" s="6" t="n"/>
+      <c r="L18" s="6" t="n"/>
+      <c r="M18" s="6" t="n"/>
+      <c r="N18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="6" t="n"/>
+      <c r="J19" s="6" t="n"/>
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="6" t="n"/>
+      <c r="M19" s="6" t="n"/>
+      <c r="N19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
+      <c r="J20" s="6" t="n"/>
+      <c r="K20" s="6" t="n"/>
+      <c r="L20" s="6" t="n"/>
+      <c r="M20" s="6" t="n"/>
+      <c r="N20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
+      <c r="I21" s="6" t="n"/>
+      <c r="J21" s="6" t="n"/>
+      <c r="K21" s="6" t="n"/>
+      <c r="L21" s="6" t="n"/>
+      <c r="M21" s="6" t="n"/>
+      <c r="N21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
+      <c r="I22" s="6" t="n"/>
+      <c r="J22" s="6" t="n"/>
+      <c r="K22" s="6" t="n"/>
+      <c r="L22" s="6" t="n"/>
+      <c r="M22" s="6" t="n"/>
+      <c r="N22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
+      <c r="I23" s="6" t="n"/>
+      <c r="J23" s="6" t="n"/>
+      <c r="K23" s="6" t="n"/>
+      <c r="L23" s="6" t="n"/>
+      <c r="M23" s="6" t="n"/>
+      <c r="N23" s="6" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="6" t="n"/>
+      <c r="H24" s="6" t="n"/>
+      <c r="I24" s="6" t="n"/>
+      <c r="J24" s="6" t="n"/>
+      <c r="K24" s="6" t="n"/>
+      <c r="L24" s="6" t="n"/>
+      <c r="M24" s="6" t="n"/>
+      <c r="N24" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="6" t="n"/>
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="6" t="n"/>
+      <c r="G25" s="6" t="n"/>
+      <c r="H25" s="6" t="n"/>
+      <c r="I25" s="6" t="n"/>
+      <c r="J25" s="6" t="n"/>
+      <c r="K25" s="6" t="n"/>
+      <c r="L25" s="6" t="n"/>
+      <c r="M25" s="6" t="n"/>
+      <c r="N25" s="6" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="6" t="n"/>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="6" t="n"/>
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="6" t="n"/>
+      <c r="I26" s="6" t="n"/>
+      <c r="J26" s="6" t="n"/>
+      <c r="K26" s="6" t="n"/>
+      <c r="L26" s="6" t="n"/>
+      <c r="M26" s="6" t="n"/>
+      <c r="N26" s="6" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="6" t="n"/>
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="6" t="n"/>
+      <c r="G27" s="6" t="n"/>
+      <c r="H27" s="6" t="n"/>
+      <c r="I27" s="6" t="n"/>
+      <c r="J27" s="6" t="n"/>
+      <c r="K27" s="6" t="n"/>
+      <c r="L27" s="6" t="n"/>
+      <c r="M27" s="6" t="n"/>
+      <c r="N27" s="6" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n"/>
+      <c r="B28" s="6" t="n"/>
+      <c r="C28" s="6" t="n"/>
+      <c r="D28" s="6" t="n"/>
+      <c r="E28" s="6" t="n"/>
+      <c r="F28" s="6" t="n"/>
+      <c r="G28" s="6" t="n"/>
+      <c r="H28" s="6" t="n"/>
+      <c r="I28" s="6" t="n"/>
+      <c r="J28" s="6" t="n"/>
+      <c r="K28" s="6" t="n"/>
+      <c r="L28" s="6" t="n"/>
+      <c r="M28" s="6" t="n"/>
+      <c r="N28" s="6" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n"/>
+      <c r="B29" s="6" t="n"/>
+      <c r="C29" s="6" t="n"/>
+      <c r="D29" s="6" t="n"/>
+      <c r="E29" s="6" t="n"/>
+      <c r="F29" s="6" t="n"/>
+      <c r="G29" s="6" t="n"/>
+      <c r="H29" s="6" t="n"/>
+      <c r="I29" s="6" t="n"/>
+      <c r="J29" s="6" t="n"/>
+      <c r="K29" s="6" t="n"/>
+      <c r="L29" s="6" t="n"/>
+      <c r="M29" s="6" t="n"/>
+      <c r="N29" s="6" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n"/>
+      <c r="B30" s="6" t="n"/>
+      <c r="C30" s="6" t="n"/>
+      <c r="D30" s="6" t="n"/>
+      <c r="E30" s="6" t="n"/>
+      <c r="F30" s="6" t="n"/>
+      <c r="G30" s="6" t="n"/>
+      <c r="H30" s="6" t="n"/>
+      <c r="I30" s="6" t="n"/>
+      <c r="J30" s="6" t="n"/>
+      <c r="K30" s="6" t="n"/>
+      <c r="L30" s="6" t="n"/>
+      <c r="M30" s="6" t="n"/>
+      <c r="N30" s="6" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n"/>
+      <c r="B31" s="6" t="n"/>
+      <c r="C31" s="6" t="n"/>
+      <c r="D31" s="6" t="n"/>
+      <c r="E31" s="6" t="n"/>
+      <c r="F31" s="6" t="n"/>
+      <c r="G31" s="6" t="n"/>
+      <c r="H31" s="6" t="n"/>
+      <c r="I31" s="6" t="n"/>
+      <c r="J31" s="6" t="n"/>
+      <c r="K31" s="6" t="n"/>
+      <c r="L31" s="6" t="n"/>
+      <c r="M31" s="6" t="n"/>
+      <c r="N31" s="6" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n"/>
+      <c r="B32" s="6" t="n"/>
+      <c r="C32" s="6" t="n"/>
+      <c r="D32" s="6" t="n"/>
+      <c r="E32" s="6" t="n"/>
+      <c r="F32" s="6" t="n"/>
+      <c r="G32" s="6" t="n"/>
+      <c r="H32" s="6" t="n"/>
+      <c r="I32" s="6" t="n"/>
+      <c r="J32" s="6" t="n"/>
+      <c r="K32" s="6" t="n"/>
+      <c r="L32" s="6" t="n"/>
+      <c r="M32" s="6" t="n"/>
+      <c r="N32" s="6" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n"/>
+      <c r="B33" s="6" t="n"/>
+      <c r="C33" s="6" t="n"/>
+      <c r="D33" s="6" t="n"/>
+      <c r="E33" s="6" t="n"/>
+      <c r="F33" s="6" t="n"/>
+      <c r="G33" s="6" t="n"/>
+      <c r="H33" s="6" t="n"/>
+      <c r="I33" s="6" t="n"/>
+      <c r="J33" s="6" t="n"/>
+      <c r="K33" s="6" t="n"/>
+      <c r="L33" s="6" t="n"/>
+      <c r="M33" s="6" t="n"/>
+      <c r="N33" s="6" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n"/>
+      <c r="B34" s="6" t="n"/>
+      <c r="C34" s="6" t="n"/>
+      <c r="D34" s="6" t="n"/>
+      <c r="E34" s="6" t="n"/>
+      <c r="F34" s="6" t="n"/>
+      <c r="G34" s="6" t="n"/>
+      <c r="H34" s="6" t="n"/>
+      <c r="I34" s="6" t="n"/>
+      <c r="J34" s="6" t="n"/>
+      <c r="K34" s="6" t="n"/>
+      <c r="L34" s="6" t="n"/>
+      <c r="M34" s="6" t="n"/>
+      <c r="N34" s="6" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n"/>
+      <c r="B35" s="6" t="n"/>
+      <c r="C35" s="6" t="n"/>
+      <c r="D35" s="6" t="n"/>
+      <c r="E35" s="6" t="n"/>
+      <c r="F35" s="6" t="n"/>
+      <c r="G35" s="6" t="n"/>
+      <c r="H35" s="6" t="n"/>
+      <c r="I35" s="6" t="n"/>
+      <c r="J35" s="6" t="n"/>
+      <c r="K35" s="6" t="n"/>
+      <c r="L35" s="6" t="n"/>
+      <c r="M35" s="6" t="n"/>
+      <c r="N35" s="6" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n"/>
+      <c r="B36" s="6" t="n"/>
+      <c r="C36" s="6" t="n"/>
+      <c r="D36" s="6" t="n"/>
+      <c r="E36" s="6" t="n"/>
+      <c r="F36" s="6" t="n"/>
+      <c r="G36" s="6" t="n"/>
+      <c r="H36" s="6" t="n"/>
+      <c r="I36" s="6" t="n"/>
+      <c r="J36" s="6" t="n"/>
+      <c r="K36" s="6" t="n"/>
+      <c r="L36" s="6" t="n"/>
+      <c r="M36" s="6" t="n"/>
+      <c r="N36" s="6" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n"/>
+      <c r="B37" s="6" t="n"/>
+      <c r="C37" s="6" t="n"/>
+      <c r="D37" s="6" t="n"/>
+      <c r="E37" s="6" t="n"/>
+      <c r="F37" s="6" t="n"/>
+      <c r="G37" s="6" t="n"/>
+      <c r="H37" s="6" t="n"/>
+      <c r="I37" s="6" t="n"/>
+      <c r="J37" s="6" t="n"/>
+      <c r="K37" s="6" t="n"/>
+      <c r="L37" s="6" t="n"/>
+      <c r="M37" s="6" t="n"/>
+      <c r="N37" s="6" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n"/>
+      <c r="B38" s="6" t="n"/>
+      <c r="C38" s="6" t="n"/>
+      <c r="D38" s="6" t="n"/>
+      <c r="E38" s="6" t="n"/>
+      <c r="F38" s="6" t="n"/>
+      <c r="G38" s="6" t="n"/>
+      <c r="H38" s="6" t="n"/>
+      <c r="I38" s="6" t="n"/>
+      <c r="J38" s="6" t="n"/>
+      <c r="K38" s="6" t="n"/>
+      <c r="L38" s="6" t="n"/>
+      <c r="M38" s="6" t="n"/>
+      <c r="N38" s="6" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n"/>
+      <c r="B39" s="6" t="n"/>
+      <c r="C39" s="6" t="n"/>
+      <c r="D39" s="6" t="n"/>
+      <c r="E39" s="6" t="n"/>
+      <c r="F39" s="6" t="n"/>
+      <c r="G39" s="6" t="n"/>
+      <c r="H39" s="6" t="n"/>
+      <c r="I39" s="6" t="n"/>
+      <c r="J39" s="6" t="n"/>
+      <c r="K39" s="6" t="n"/>
+      <c r="L39" s="6" t="n"/>
+      <c r="M39" s="6" t="n"/>
+      <c r="N39" s="6" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n"/>
+      <c r="B40" s="6" t="n"/>
+      <c r="C40" s="6" t="n"/>
+      <c r="D40" s="6" t="n"/>
+      <c r="E40" s="6" t="n"/>
+      <c r="F40" s="6" t="n"/>
+      <c r="G40" s="6" t="n"/>
+      <c r="H40" s="6" t="n"/>
+      <c r="I40" s="6" t="n"/>
+      <c r="J40" s="6" t="n"/>
+      <c r="K40" s="6" t="n"/>
+      <c r="L40" s="6" t="n"/>
+      <c r="M40" s="6" t="n"/>
+      <c r="N40" s="6" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n"/>
+      <c r="B41" s="6" t="n"/>
+      <c r="C41" s="6" t="n"/>
+      <c r="D41" s="6" t="n"/>
+      <c r="E41" s="6" t="n"/>
+      <c r="F41" s="6" t="n"/>
+      <c r="G41" s="6" t="n"/>
+      <c r="H41" s="6" t="n"/>
+      <c r="I41" s="6" t="n"/>
+      <c r="J41" s="6" t="n"/>
+      <c r="K41" s="6" t="n"/>
+      <c r="L41" s="6" t="n"/>
+      <c r="M41" s="6" t="n"/>
+      <c r="N41" s="6" t="n"/>
     </row>
   </sheetData>
+  <dataValidations count="4">
+    <dataValidation sqref="A2:A41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not one of the choices" error="Choose one of the listed answers." type="list" errorStyle="information">
+      <formula1>Alternatives!$A$2:$A$100</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not one of the choices" error="Choose one of the listed answers." type="list" errorStyle="stop">
+      <formula1>"RDT&amp;E,Procurement,MILCON,O&amp;S,Disposal"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not one of the choices" error="Choose one of the listed answers." type="list" errorStyle="information">
+      <formula1>"uniform,front,back,bell"</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not one of the choices" error="Choose one of the listed answers." type="list" errorStyle="stop">
+      <formula1>"triangular,pert,uniform"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FFC000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1223,49 +2011,206 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Alternative</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Line</t>
         </is>
       </c>
-      <c r="C1" s="1" t="n">
+      <c r="C1" s="5" t="n">
         <v>2061</v>
       </c>
-      <c r="D1" s="1" t="n">
+      <c r="D1" s="5" t="n">
         <v>2062</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>New development</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Disposal</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="6" t="n">
         <v>60</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="6" t="n">
         <v>60</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="6" t="n"/>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n"/>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="6" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="6" t="n"/>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="6" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="6" t="n"/>
+    </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not one of the choices" error="Choose one of the listed answers." type="list" errorStyle="information">
+      <formula1>Alternatives!$A$2:$A$100</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FFC000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -1277,127 +2222,137 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Setting</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Base Year</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="6" t="n">
         <v>2026</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Discount Rate</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="6" t="n">
         <v>0.02</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Inflation Rate</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="6" t="n">
         <v>0.021</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>BY2026 $M</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Basis</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>pv</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Status Quo</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Keep current system</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Iterations</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="6" t="n">
         <v>20000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Seed</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="6" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Invented numbers, for illustration only: three ways to replace an ageing sensor, and keeping it, in BY2026 $M.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not one of the choices" error="Choose one of the listed answers." type="list" errorStyle="information">
+      <formula1>"pv,by,ty"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not one of the choices" error="Choose one of the listed answers." type="list" errorStyle="information">
+      <formula1>Alternatives!$A$2:$A$100</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00A6A6A6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1405,72 +2360,139 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>How to fill in this workbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Yellow cells</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Yours to fill in. The example rows are there to show the layout: type over them, and add more rows in the yellow space below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Dark blue heading</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>A column that must be filled in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Light blue heading</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>An optional column: leave it blank if it doesn't apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Grey cells</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Labels: leave them as they are.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Hover over a heading</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>A note says what goes in that column, in what units, with an example. A small arrow in a cell means a drop-down list of the allowed answers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>Sheet or topic</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>What to put there</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>What this is</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>The alternatives for a capability and their costs over the life cycle, for an analysis of alternatives: ce-core aoa --spec &lt;this file&gt;.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Alternatives sheet</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>One row per alternative. Effectiveness is optional, on any scale that is the same for all of them. Correlation (default 0.3) is how much its cost lines overrun together.</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Lines sheet</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>One cost line per row, naming its Alternative. Give its cost one of three ways: a Total spread over Years from a Start Year (Profile uniform, front, back or bell); an Annual Amount from a First Year to a Last Year; or a row on the Phased sheet with the amount in each year.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Uncertainty</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Low, Most Likely and High Factor multiply the line: 0.9, 1.0, 1.4 means 10% under to 40% over. Leave them blank for a line with no uncertainty.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Settings sheet</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Base Year is the constant-dollar year. Discount Rate and Inflation Rate are annual (0.02 for 2%). Basis is by, ty or pv: which dollars to compare on. Status Quo names the alternative the others are measured against in the economic analysis: what each costs up front, what it saves, whether it pays back and when.</t>
         </is>

</xml_diff>